<commit_message>
feat: migrate persistence to postgres and redis
</commit_message>
<xml_diff>
--- a/Example/demo-os.xlsx
+++ b/Example/demo-os.xlsx
@@ -523,7 +523,7 @@
         <v>POLO-01</v>
       </c>
       <c r="G5" t="str">
-        <v>F0001</v>
+        <v/>
       </c>
       <c r="H5" t="str">
         <v/>
@@ -575,7 +575,7 @@
         <v>POLO-01</v>
       </c>
       <c r="G7" t="str">
-        <v>F0001</v>
+        <v/>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -627,7 +627,7 @@
         <v>POLO-01</v>
       </c>
       <c r="G9" t="str">
-        <v>F0001</v>
+        <v/>
       </c>
       <c r="H9" t="str">
         <v/>

</xml_diff>

<commit_message>
Tipo de Servico segue os tipos do formulario FFR
Substitui o enum TipoServico (categorias de agua + Outros) pelos 6 tipos
oficiais do Formulario FFR v2026_04_06 (aba "FFR") + "Outros" como catch-all:
Rede/ramal de agua, Cavalete/hidrometro, Rede/ramal de esgoto, Desobstrucao,
Reposicao piso/passeio/..., Reposicao asfaltica.

- schema.prisma + migracao: converte OS existentes (reclassifica pela
  Descricao TSS, com fallback do enum antigo).
- os-labels, importacao (classificador), grupos-ffr (tipos + fallback) e o
  dropdown da Fila atualizados para os novos tipos.
- demo-os.ts + Example/demo-os.xlsx (novo scripts/gen-demo-xlsx.ts) cobrindo
  as novas categorias.
- Testes atualizados; typecheck limpo, 258 passando.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Example/demo-os.xlsx
+++ b/Example/demo-os.xlsx
@@ -439,7 +439,7 @@
         <v>Cidade Teste</v>
       </c>
       <c r="E2" t="str">
-        <v>LigacaoAgua</v>
+        <v>RedeRamalAgua</v>
       </c>
       <c r="F2" t="str">
         <v>POLO-01</v>
@@ -465,7 +465,7 @@
         <v>Cidade Teste</v>
       </c>
       <c r="E3" t="str">
-        <v>Vistoria</v>
+        <v>Outros</v>
       </c>
       <c r="F3" t="str">
         <v>POLO-01</v>
@@ -491,7 +491,7 @@
         <v>Cidade Teste</v>
       </c>
       <c r="E4" t="str">
-        <v>ReparoRede</v>
+        <v>RedeRamalEsgoto</v>
       </c>
       <c r="F4" t="str">
         <v>POLO-01</v>
@@ -517,7 +517,7 @@
         <v>Cidade Teste</v>
       </c>
       <c r="E5" t="str">
-        <v>TrocaHidrometro</v>
+        <v>CavaleteHidrometro</v>
       </c>
       <c r="F5" t="str">
         <v>POLO-01</v>
@@ -543,7 +543,7 @@
         <v>Cidade Teste</v>
       </c>
       <c r="E6" t="str">
-        <v>ReligacaoAgua</v>
+        <v>Desobstrucao</v>
       </c>
       <c r="F6" t="str">
         <v>POLO-01</v>
@@ -569,7 +569,7 @@
         <v>Cidade Teste</v>
       </c>
       <c r="E7" t="str">
-        <v>CorteAgua</v>
+        <v>CavaleteHidrometro</v>
       </c>
       <c r="F7" t="str">
         <v>POLO-01</v>
@@ -595,7 +595,7 @@
         <v>Cidade Teste</v>
       </c>
       <c r="E8" t="str">
-        <v>Outros</v>
+        <v>ReposicaoPiso</v>
       </c>
       <c r="F8" t="str">
         <v>POLO-01</v>
@@ -621,7 +621,7 @@
         <v>Cidade Teste</v>
       </c>
       <c r="E9" t="str">
-        <v>Vistoria</v>
+        <v>ReposicaoAsfaltica</v>
       </c>
       <c r="F9" t="str">
         <v>POLO-01</v>

</xml_diff>